<commit_message>
basic update, based on new TWONTO file
</commit_message>
<xml_diff>
--- a/Avantis Mapping/SPARQL_class.xlsx
+++ b/Avantis Mapping/SPARQL_class.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\medney\Documents\GitHub\TWONTO\Avantis Mapping\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCAAEC70-EC44-4659-87F8-055AABA5EC47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D1EC3E0-1B2B-4F29-AEB8-8B1AE883ACB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{716C0CF8-2E33-46F2-BE6F-578AC5702A19}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{716C0CF8-2E33-46F2-BE6F-578AC5702A19}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="251">
   <si>
     <t>TWONTO</t>
   </si>
@@ -750,9 +750,6 @@
     <t>http://www.toronto.ca/TWONTO#blower</t>
   </si>
   <si>
-    <t>http://www.toronto.ca/TWONTO#fuel_burning_heater</t>
-  </si>
-  <si>
     <t>http://www.toronto.ca/TWONTO#network_panel</t>
   </si>
   <si>
@@ -763,6 +760,45 @@
   </si>
   <si>
     <t>Silencer</t>
+  </si>
+  <si>
+    <t>http://www.toronto.ca/TWONTO#venturi_flow_sensor_element</t>
+  </si>
+  <si>
+    <t>Remote Transmission Unit</t>
+  </si>
+  <si>
+    <t>http://www.toronto.ca/TWONTO#network_switch</t>
+  </si>
+  <si>
+    <t>Network Switch</t>
+  </si>
+  <si>
+    <t>http://www.toronto.ca/TWONTO#burner_-_component_of_asset</t>
+  </si>
+  <si>
+    <t>http://www.toronto.ca/TWONTO#flowmeter</t>
+  </si>
+  <si>
+    <t>Meter</t>
+  </si>
+  <si>
+    <t>http://www.toronto.ca/TWONTO#weight_scale</t>
+  </si>
+  <si>
+    <t>Weigh Scale</t>
+  </si>
+  <si>
+    <t>http://www.toronto.ca/TWONTO#process_controller</t>
+  </si>
+  <si>
+    <t>http://www.toronto.ca/TWONTO#cable_segment</t>
+  </si>
+  <si>
+    <t>Electrical Power Line</t>
+  </si>
+  <si>
+    <t>http://www.toronto.ca/TWONTO#equipment_chamber_or_access_chamber</t>
   </si>
 </sst>
 </file>
@@ -923,8 +959,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2F59859A-FBE4-49A6-B6BA-B68B6E359698}" name="Table1" displayName="Table1" ref="A2:B123" totalsRowShown="0" headerRowDxfId="3">
-  <autoFilter ref="A2:B123" xr:uid="{2F59859A-FBE4-49A6-B6BA-B68B6E359698}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2F59859A-FBE4-49A6-B6BA-B68B6E359698}" name="Table1" displayName="Table1" ref="A2:B126" totalsRowShown="0" headerRowDxfId="3">
+  <autoFilter ref="A2:B126" xr:uid="{2F59859A-FBE4-49A6-B6BA-B68B6E359698}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:B3">
     <sortCondition ref="B2:B3"/>
   </sortState>
@@ -1247,19 +1283,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C799550E-49B1-4512-9CC1-86876BA1337E}">
-  <dimension ref="A1:B123"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B126"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="69.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="26.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="69.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="165" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" ht="159.5" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1267,7 +1303,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>104</v>
       </c>
@@ -1275,7 +1311,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>233</v>
       </c>
@@ -1283,7 +1319,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>105</v>
       </c>
@@ -1291,7 +1327,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>106</v>
       </c>
@@ -1299,7 +1335,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>107</v>
       </c>
@@ -1307,7 +1343,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>233</v>
       </c>
@@ -1315,23 +1351,23 @@
         <v>88</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>234</v>
+        <v>108</v>
       </c>
       <c r="B9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>109</v>
+      </c>
+      <c r="B10" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>108</v>
-      </c>
-      <c r="B10" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>110</v>
       </c>
@@ -1339,7 +1375,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>111</v>
       </c>
@@ -1347,7 +1383,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>112</v>
       </c>
@@ -1355,7 +1391,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>113</v>
       </c>
@@ -1363,7 +1399,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>114</v>
       </c>
@@ -1371,7 +1407,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>115</v>
       </c>
@@ -1379,7 +1415,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>199</v>
       </c>
@@ -1387,7 +1423,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>116</v>
       </c>
@@ -1395,7 +1431,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>117</v>
       </c>
@@ -1403,7 +1439,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>118</v>
       </c>
@@ -1411,7 +1447,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>119</v>
       </c>
@@ -1419,7 +1455,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>120</v>
       </c>
@@ -1427,7 +1463,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>121</v>
       </c>
@@ -1435,7 +1471,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>122</v>
       </c>
@@ -1443,7 +1479,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>201</v>
       </c>
@@ -1451,7 +1487,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>123</v>
       </c>
@@ -1459,7 +1495,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>124</v>
       </c>
@@ -1467,7 +1503,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>125</v>
       </c>
@@ -1475,7 +1511,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>126</v>
       </c>
@@ -1483,7 +1519,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>127</v>
       </c>
@@ -1491,7 +1527,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>128</v>
       </c>
@@ -1499,7 +1535,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>129</v>
       </c>
@@ -1507,7 +1543,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>130</v>
       </c>
@@ -1515,7 +1551,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>225</v>
       </c>
@@ -1523,7 +1559,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>131</v>
       </c>
@@ -1531,7 +1567,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>132</v>
       </c>
@@ -1539,7 +1575,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>133</v>
       </c>
@@ -1547,7 +1583,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>134</v>
       </c>
@@ -1555,47 +1591,47 @@
         <v>22</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
+        <v>238</v>
+      </c>
+      <c r="B39" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
         <v>135</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B40" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
         <v>136</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B41" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
         <v>137</v>
       </c>
-      <c r="B41" t="s">
+      <c r="B42" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
         <v>138</v>
       </c>
-      <c r="B42" t="s">
+      <c r="B43" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>139</v>
-      </c>
-      <c r="B43" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>140</v>
       </c>
@@ -1603,7 +1639,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>141</v>
       </c>
@@ -1611,7 +1647,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>219</v>
       </c>
@@ -1619,7 +1655,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>142</v>
       </c>
@@ -1627,7 +1663,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>143</v>
       </c>
@@ -1635,601 +1671,625 @@
         <v>29</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
+        <v>210</v>
+      </c>
+      <c r="B49" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
         <v>144</v>
       </c>
-      <c r="B49" t="s">
+      <c r="B50" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
         <v>211</v>
       </c>
-      <c r="B50" t="s">
+      <c r="B51" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
         <v>145</v>
       </c>
-      <c r="B51" t="s">
+      <c r="B52" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
         <v>146</v>
       </c>
-      <c r="B52" t="s">
+      <c r="B53" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
         <v>147</v>
       </c>
-      <c r="B53" t="s">
+      <c r="B54" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
         <v>148</v>
       </c>
-      <c r="B54" t="s">
+      <c r="B55" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
         <v>149</v>
       </c>
-      <c r="B55" t="s">
+      <c r="B56" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A57" t="s">
         <v>150</v>
       </c>
-      <c r="B56" t="s">
+      <c r="B57" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A58" t="s">
         <v>151</v>
       </c>
-      <c r="B57" t="s">
+      <c r="B58" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A59" t="s">
         <v>152</v>
       </c>
-      <c r="B58" t="s">
+      <c r="B59" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A60" t="s">
         <v>153</v>
       </c>
-      <c r="B59" t="s">
+      <c r="B60" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A61" t="s">
         <v>154</v>
       </c>
-      <c r="B60" t="s">
+      <c r="B61" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
         <v>115</v>
       </c>
-      <c r="B61" t="s">
+      <c r="B62" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
         <v>217</v>
       </c>
-      <c r="B62" t="s">
+      <c r="B63" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A64" t="s">
         <v>155</v>
       </c>
-      <c r="B63" t="s">
+      <c r="B64" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A65" t="s">
         <v>156</v>
       </c>
-      <c r="B64" t="s">
+      <c r="B65" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A66" t="s">
         <v>157</v>
       </c>
-      <c r="B65" t="s">
+      <c r="B66" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A67" t="s">
         <v>158</v>
       </c>
-      <c r="B66" t="s">
+      <c r="B67" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A68" t="s">
         <v>159</v>
       </c>
-      <c r="B67" t="s">
+      <c r="B68" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
+        <v>240</v>
+      </c>
+      <c r="B69" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A70" t="s">
         <v>160</v>
       </c>
-      <c r="B68" t="s">
+      <c r="B70" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
         <v>161</v>
       </c>
-      <c r="B69" t="s">
+      <c r="B71" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A72" t="s">
         <v>162</v>
       </c>
-      <c r="B70" t="s">
+      <c r="B72" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
         <v>112</v>
       </c>
-      <c r="B71" t="s">
+      <c r="B73" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
-        <v>131</v>
-      </c>
-      <c r="B72" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A74" t="s">
         <v>163</v>
       </c>
-      <c r="B73" t="s">
+      <c r="B74" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A74" t="s">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A75" t="s">
+        <v>242</v>
+      </c>
+      <c r="B75" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A76" t="s">
         <v>164</v>
       </c>
-      <c r="B74" t="s">
+      <c r="B76" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A77" t="s">
+        <v>243</v>
+      </c>
+      <c r="B77" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A78" t="s">
         <v>165</v>
       </c>
-      <c r="B75" t="s">
+      <c r="B78" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A79" t="s">
         <v>166</v>
       </c>
-      <c r="B76" t="s">
+      <c r="B79" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A77" t="s">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A80" t="s">
         <v>204</v>
       </c>
-      <c r="B77" t="s">
+      <c r="B80" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A78" t="s">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A81" t="s">
         <v>214</v>
       </c>
-      <c r="B78" t="s">
+      <c r="B81" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A79" t="s">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A82" t="s">
         <v>167</v>
       </c>
-      <c r="B79" t="s">
+      <c r="B82" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A80" t="s">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A83" t="s">
         <v>168</v>
       </c>
-      <c r="B80" t="s">
+      <c r="B83" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A81" t="s">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A84" t="s">
         <v>169</v>
       </c>
-      <c r="B81" t="s">
+      <c r="B84" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A82" t="s">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A85" t="s">
+        <v>245</v>
+      </c>
+      <c r="B85" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A86" t="s">
         <v>170</v>
       </c>
-      <c r="B82" t="s">
+      <c r="B86" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A83" t="s">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A87" t="s">
         <v>229</v>
       </c>
-      <c r="B83" t="s">
+      <c r="B87" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A84" t="s">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A88" t="s">
         <v>171</v>
       </c>
-      <c r="B84" t="s">
+      <c r="B88" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A85" t="s">
-        <v>172</v>
-      </c>
-      <c r="B85" t="s">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A89" t="s">
+        <v>173</v>
+      </c>
+      <c r="B89" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A90" t="s">
+        <v>174</v>
+      </c>
+      <c r="B90" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A91" t="s">
+        <v>210</v>
+      </c>
+      <c r="B91" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A92" t="s">
+        <v>175</v>
+      </c>
+      <c r="B92" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A93" t="s">
+        <v>176</v>
+      </c>
+      <c r="B93" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A94" t="s">
+        <v>177</v>
+      </c>
+      <c r="B94" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A95" t="s">
+        <v>227</v>
+      </c>
+      <c r="B95" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A96" t="s">
+        <v>205</v>
+      </c>
+      <c r="B96" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A97" t="s">
+        <v>178</v>
+      </c>
+      <c r="B97" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A98" t="s">
+        <v>179</v>
+      </c>
+      <c r="B98" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A99" t="s">
+        <v>180</v>
+      </c>
+      <c r="B99" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A100" t="s">
+        <v>181</v>
+      </c>
+      <c r="B100" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A101" t="s">
+        <v>182</v>
+      </c>
+      <c r="B101" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A102" t="s">
+        <v>184</v>
+      </c>
+      <c r="B102" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A103" t="s">
+        <v>185</v>
+      </c>
+      <c r="B103" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A104" t="s">
+        <v>247</v>
+      </c>
+      <c r="B104" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A105" t="s">
+        <v>154</v>
+      </c>
+      <c r="B105" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A106" t="s">
+        <v>186</v>
+      </c>
+      <c r="B106" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A107" t="s">
+        <v>113</v>
+      </c>
+      <c r="B107" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A108" t="s">
+        <v>187</v>
+      </c>
+      <c r="B108" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A109" t="s">
+        <v>236</v>
+      </c>
+      <c r="B109" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A110" t="s">
+        <v>231</v>
+      </c>
+      <c r="B110" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A111" t="s">
+        <v>188</v>
+      </c>
+      <c r="B111" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A112" t="s">
+        <v>248</v>
+      </c>
+      <c r="B112" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A113" t="s">
+        <v>189</v>
+      </c>
+      <c r="B113" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A114" t="s">
+        <v>190</v>
+      </c>
+      <c r="B114" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A115" t="s">
+        <v>234</v>
+      </c>
+      <c r="B115" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A116" t="s">
+        <v>192</v>
+      </c>
+      <c r="B116" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A117" t="s">
+        <v>193</v>
+      </c>
+      <c r="B117" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A118" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A119" t="s">
+        <v>221</v>
+      </c>
+      <c r="B119" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A120" t="s">
+        <v>195</v>
+      </c>
+      <c r="B120" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A121" t="s">
+        <v>196</v>
+      </c>
+      <c r="B121" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A122" t="s">
+        <v>197</v>
+      </c>
+      <c r="B122" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A123" t="s">
+        <v>223</v>
+      </c>
+      <c r="B123" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A124" t="s">
+        <v>159</v>
+      </c>
+      <c r="B124" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A125" t="s">
+        <v>250</v>
+      </c>
+      <c r="B125" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A86" t="s">
-        <v>173</v>
-      </c>
-      <c r="B86" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A87" t="s">
-        <v>174</v>
-      </c>
-      <c r="B87" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A88" t="s">
-        <v>210</v>
-      </c>
-      <c r="B88" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A89" t="s">
-        <v>175</v>
-      </c>
-      <c r="B89" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A90" t="s">
-        <v>176</v>
-      </c>
-      <c r="B90" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A91" t="s">
-        <v>177</v>
-      </c>
-      <c r="B91" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A92" t="s">
-        <v>227</v>
-      </c>
-      <c r="B92" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A93" t="s">
-        <v>205</v>
-      </c>
-      <c r="B93" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A94" t="s">
-        <v>178</v>
-      </c>
-      <c r="B94" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A95" t="s">
-        <v>179</v>
-      </c>
-      <c r="B95" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A96" t="s">
-        <v>180</v>
-      </c>
-      <c r="B96" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A97" t="s">
-        <v>181</v>
-      </c>
-      <c r="B97" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A98" t="s">
-        <v>182</v>
-      </c>
-      <c r="B98" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A99" t="s">
-        <v>183</v>
-      </c>
-      <c r="B99" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A100" t="s">
-        <v>184</v>
-      </c>
-      <c r="B100" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A101" t="s">
-        <v>185</v>
-      </c>
-      <c r="B101" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A102" t="s">
-        <v>154</v>
-      </c>
-      <c r="B102" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A103" t="s">
-        <v>186</v>
-      </c>
-      <c r="B103" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A104" t="s">
-        <v>113</v>
-      </c>
-      <c r="B104" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A105" t="s">
-        <v>187</v>
-      </c>
-      <c r="B105" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A106" t="s">
-        <v>231</v>
-      </c>
-      <c r="B106" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A107" t="s">
-        <v>188</v>
-      </c>
-      <c r="B107" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A108" t="s">
-        <v>189</v>
-      </c>
-      <c r="B108" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A109" t="s">
-        <v>190</v>
-      </c>
-      <c r="B109" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A110" t="s">
-        <v>191</v>
-      </c>
-      <c r="B110" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A111" t="s">
-        <v>235</v>
-      </c>
-      <c r="B111" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A112" t="s">
-        <v>192</v>
-      </c>
-      <c r="B112" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A113" t="s">
-        <v>193</v>
-      </c>
-      <c r="B113" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A114" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A115" t="s">
-        <v>221</v>
-      </c>
-      <c r="B115" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A116" t="s">
-        <v>195</v>
-      </c>
-      <c r="B116" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A117" t="s">
-        <v>206</v>
-      </c>
-      <c r="B117" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A118" t="s">
-        <v>196</v>
-      </c>
-      <c r="B118" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A119" t="s">
-        <v>197</v>
-      </c>
-      <c r="B119" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A120" t="s">
-        <v>223</v>
-      </c>
-      <c r="B120" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A121" t="s">
-        <v>159</v>
-      </c>
-      <c r="B121" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A122" t="s">
+    <row r="126" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A126" t="s">
         <v>198</v>
       </c>
-      <c r="B122" t="s">
+      <c r="B126" t="s">
         <v>76</v>
-      </c>
-    </row>
-    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A123" t="s">
-        <v>237</v>
-      </c>
-      <c r="B123" t="s">
-        <v>238</v>
       </c>
     </row>
   </sheetData>
@@ -2244,13 +2304,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4884BCF2-D0BF-43AF-A366-0080E3AC3682}">
   <dimension ref="C3:D110"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="3" max="3" width="73.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.140625" customWidth="1"/>
+    <col min="3" max="3" width="73.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C3" s="3" t="s">
         <v>0</v>
       </c>
@@ -2258,7 +2318,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C4" t="s">
         <v>170</v>
       </c>
@@ -2266,7 +2326,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="5" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C5" t="s">
         <v>115</v>
       </c>
@@ -2274,7 +2334,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="6" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C6" t="s">
         <v>178</v>
       </c>
@@ -2282,7 +2342,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="7" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C7" t="s">
         <v>175</v>
       </c>
@@ -2290,7 +2350,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="8" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C8" t="s">
         <v>105</v>
       </c>
@@ -2298,7 +2358,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C9" t="s">
         <v>205</v>
       </c>
@@ -2306,7 +2366,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="10" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C10" t="s">
         <v>188</v>
       </c>
@@ -2314,7 +2374,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="11" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C11" t="s">
         <v>130</v>
       </c>
@@ -2322,7 +2382,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="12" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C12" t="s">
         <v>126</v>
       </c>
@@ -2330,7 +2390,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C13" t="s">
         <v>197</v>
       </c>
@@ -2338,7 +2398,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="14" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C14" t="s">
         <v>209</v>
       </c>
@@ -2346,7 +2406,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="15" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C15" t="s">
         <v>167</v>
       </c>
@@ -2354,7 +2414,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="16" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C16" t="s">
         <v>129</v>
       </c>
@@ -2362,7 +2422,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="17" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C17" t="s">
         <v>113</v>
       </c>
@@ -2370,7 +2430,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="18" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C18" t="s">
         <v>139</v>
       </c>
@@ -2378,7 +2438,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="19" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C19" t="s">
         <v>190</v>
       </c>
@@ -2386,7 +2446,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="20" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C20" t="s">
         <v>124</v>
       </c>
@@ -2394,7 +2454,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="21" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C21" t="s">
         <v>172</v>
       </c>
@@ -2402,7 +2462,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="22" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C22" t="s">
         <v>122</v>
       </c>
@@ -2410,7 +2470,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="23" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C23" t="s">
         <v>195</v>
       </c>
@@ -2418,7 +2478,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="24" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C24" t="s">
         <v>159</v>
       </c>
@@ -2426,7 +2486,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="25" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C25" t="s">
         <v>107</v>
       </c>
@@ -2434,7 +2494,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C26" t="s">
         <v>158</v>
       </c>
@@ -2442,7 +2502,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="27" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C27" t="s">
         <v>166</v>
       </c>
@@ -2450,7 +2510,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="28" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C28" t="s">
         <v>146</v>
       </c>
@@ -2458,7 +2518,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="29" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C29" t="s">
         <v>147</v>
       </c>
@@ -2466,7 +2526,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="30" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C30" t="s">
         <v>140</v>
       </c>
@@ -2474,7 +2534,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="31" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C31" t="s">
         <v>128</v>
       </c>
@@ -2482,7 +2542,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C32" t="s">
         <v>117</v>
       </c>
@@ -2490,7 +2550,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="33" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C33" t="s">
         <v>191</v>
       </c>
@@ -2498,7 +2558,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="34" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C34" t="s">
         <v>145</v>
       </c>
@@ -2506,7 +2566,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="35" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C35" t="s">
         <v>198</v>
       </c>
@@ -2514,7 +2574,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="36" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C36" t="s">
         <v>133</v>
       </c>
@@ -2522,7 +2582,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="37" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C37" t="s">
         <v>121</v>
       </c>
@@ -2530,7 +2590,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="38" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C38" t="s">
         <v>143</v>
       </c>
@@ -2538,7 +2598,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="39" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C39" t="s">
         <v>108</v>
       </c>
@@ -2546,7 +2606,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="40" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C40" t="s">
         <v>125</v>
       </c>
@@ -2554,7 +2614,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="41" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C41" t="s">
         <v>120</v>
       </c>
@@ -2562,7 +2622,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="42" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C42" t="s">
         <v>114</v>
       </c>
@@ -2570,7 +2630,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="43" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C43" t="s">
         <v>112</v>
       </c>
@@ -2578,7 +2638,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="44" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C44" t="s">
         <v>206</v>
       </c>
@@ -2586,7 +2646,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="45" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C45" t="s">
         <v>162</v>
       </c>
@@ -2594,7 +2654,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="46" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C46" t="s">
         <v>169</v>
       </c>
@@ -2602,7 +2662,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="47" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C47" t="s">
         <v>209</v>
       </c>
@@ -2610,7 +2670,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="48" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C48" t="s">
         <v>168</v>
       </c>
@@ -2618,7 +2678,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="49" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C49" t="s">
         <v>144</v>
       </c>
@@ -2626,7 +2686,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="50" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C50" t="s">
         <v>180</v>
       </c>
@@ -2634,7 +2694,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="51" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C51" t="s">
         <v>118</v>
       </c>
@@ -2642,7 +2702,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="52" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="52" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C52" t="s">
         <v>150</v>
       </c>
@@ -2650,7 +2710,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="53" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="53" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C53" t="s">
         <v>104</v>
       </c>
@@ -2658,7 +2718,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="54" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="54" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C54" t="s">
         <v>134</v>
       </c>
@@ -2666,7 +2726,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="55" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="55" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C55" t="s">
         <v>148</v>
       </c>
@@ -2674,7 +2734,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="56" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="56" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C56" t="s">
         <v>182</v>
       </c>
@@ -2682,7 +2742,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="57" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="57" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C57" t="s">
         <v>109</v>
       </c>
@@ -2690,7 +2750,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="58" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="58" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C58" t="s">
         <v>141</v>
       </c>
@@ -2698,7 +2758,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="59" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="59" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C59" t="s">
         <v>137</v>
       </c>
@@ -2706,7 +2766,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="60" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="60" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C60" t="s">
         <v>196</v>
       </c>
@@ -2714,7 +2774,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="61" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="61" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C61" t="s">
         <v>193</v>
       </c>
@@ -2722,7 +2782,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="62" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="62" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C62" t="s">
         <v>189</v>
       </c>
@@ -2730,7 +2790,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="63" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="63" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C63" t="s">
         <v>173</v>
       </c>
@@ -2738,7 +2798,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="64" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="64" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C64" t="s">
         <v>111</v>
       </c>
@@ -2746,7 +2806,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="65" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="65" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C65" t="s">
         <v>204</v>
       </c>
@@ -2754,7 +2814,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="66" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="66" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C66" t="s">
         <v>153</v>
       </c>
@@ -2762,7 +2822,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="67" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="67" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C67" t="s">
         <v>115</v>
       </c>
@@ -2770,7 +2830,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="68" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="68" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C68" t="s">
         <v>160</v>
       </c>
@@ -2778,7 +2838,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="69" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="69" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C69" t="s">
         <v>123</v>
       </c>
@@ -2786,7 +2846,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="70" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="70" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C70" t="s">
         <v>151</v>
       </c>
@@ -2794,7 +2854,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="71" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="71" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C71" t="s">
         <v>181</v>
       </c>
@@ -2802,7 +2862,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="72" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="72" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C72" t="s">
         <v>136</v>
       </c>
@@ -2810,7 +2870,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="73" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="73" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C73" t="s">
         <v>165</v>
       </c>
@@ -2818,7 +2878,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="74" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="74" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C74" t="s">
         <v>152</v>
       </c>
@@ -2826,7 +2886,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="75" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="75" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C75" t="s">
         <v>110</v>
       </c>
@@ -2834,7 +2894,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="76" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="76" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C76" t="s">
         <v>201</v>
       </c>
@@ -2842,7 +2902,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="77" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="77" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C77" t="s">
         <v>186</v>
       </c>
@@ -2850,7 +2910,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="78" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="78" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C78" t="s">
         <v>119</v>
       </c>
@@ -2858,7 +2918,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="79" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="79" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C79" t="s">
         <v>171</v>
       </c>
@@ -2866,7 +2926,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="80" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="80" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C80" t="s">
         <v>210</v>
       </c>
@@ -2874,7 +2934,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="81" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="81" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C81" t="s">
         <v>199</v>
       </c>
@@ -2882,7 +2942,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="82" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="82" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C82" t="s">
         <v>176</v>
       </c>
@@ -2890,7 +2950,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="83" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="83" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C83" t="s">
         <v>156</v>
       </c>
@@ -2898,7 +2958,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="84" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="84" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C84" t="s">
         <v>154</v>
       </c>
@@ -2906,7 +2966,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="85" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="85" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C85" t="s">
         <v>131</v>
       </c>
@@ -2914,7 +2974,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="86" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="86" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C86" t="s">
         <v>138</v>
       </c>
@@ -2922,7 +2982,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="87" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="87" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C87" t="s">
         <v>161</v>
       </c>
@@ -2930,7 +2990,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="88" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="88" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C88" t="s">
         <v>164</v>
       </c>
@@ -2938,7 +2998,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="89" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="89" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C89" t="s">
         <v>185</v>
       </c>
@@ -2946,7 +3006,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="90" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="90" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C90" t="s">
         <v>142</v>
       </c>
@@ -2954,7 +3014,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="91" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="91" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C91" t="s">
         <v>127</v>
       </c>
@@ -2962,7 +3022,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="92" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="92" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C92" t="s">
         <v>113</v>
       </c>
@@ -2970,7 +3030,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="93" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="93" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C93" t="s">
         <v>177</v>
       </c>
@@ -2978,7 +3038,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="94" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="94" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C94" t="s">
         <v>159</v>
       </c>
@@ -2986,7 +3046,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="95" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="95" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C95" t="s">
         <v>157</v>
       </c>
@@ -2994,7 +3054,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="96" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="96" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C96" t="s">
         <v>163</v>
       </c>
@@ -3002,7 +3062,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="97" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="97" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C97" t="s">
         <v>155</v>
       </c>
@@ -3010,7 +3070,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="98" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="98" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C98" t="s">
         <v>132</v>
       </c>
@@ -3018,7 +3078,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="99" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="99" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C99" t="s">
         <v>135</v>
       </c>
@@ -3026,7 +3086,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="100" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="100" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C100" t="s">
         <v>179</v>
       </c>
@@ -3034,7 +3094,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="101" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="101" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C101" t="s">
         <v>106</v>
       </c>
@@ -3042,7 +3102,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="102" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="102" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C102" t="s">
         <v>184</v>
       </c>
@@ -3050,7 +3110,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="103" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="103" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C103" t="s">
         <v>187</v>
       </c>
@@ -3058,7 +3118,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="104" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="104" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C104" t="s">
         <v>192</v>
       </c>
@@ -3066,7 +3126,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="105" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="105" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C105" t="s">
         <v>116</v>
       </c>
@@ -3074,7 +3134,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="106" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="106" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C106" t="s">
         <v>149</v>
       </c>
@@ -3082,7 +3142,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="107" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="107" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C107" t="s">
         <v>112</v>
       </c>
@@ -3090,7 +3150,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="108" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="108" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C108" t="s">
         <v>183</v>
       </c>
@@ -3098,7 +3158,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="109" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="109" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C109" t="s">
         <v>174</v>
       </c>
@@ -3106,7 +3166,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="110" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="110" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C110" t="s">
         <v>194</v>
       </c>

</xml_diff>

<commit_message>
multiple files updates, include ML model completion
</commit_message>
<xml_diff>
--- a/Avantis Mapping/SPARQL_class.xlsx
+++ b/Avantis Mapping/SPARQL_class.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\medney\Documents\GitHub\TWONTO\Avantis Mapping\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFF17061-BEB7-4638-BF49-997AB6F2C7D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3D4C155-79E7-4B20-B76E-76F3A9BDD2A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{716C0CF8-2E33-46F2-BE6F-578AC5702A19}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{716C0CF8-2E33-46F2-BE6F-578AC5702A19}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="240">
   <si>
     <t>TWONTO</t>
   </si>
@@ -759,6 +759,12 @@
     ?sub tw:is_equivalent_to_Avantis_class ?object .
     FILTER NOT EXISTS { ?sub owl:deprecated "true"^^xsd:boolean }
 }</t>
+  </si>
+  <si>
+    <t>http://www.toronto.ca/TWONTO#00920</t>
+  </si>
+  <si>
+    <t>Office Equipment</t>
   </si>
 </sst>
 </file>
@@ -857,8 +863,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2F59859A-FBE4-49A6-B6BA-B68B6E359698}" name="Table1" displayName="Table1" ref="A2:B123" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A2:B123" xr:uid="{2F59859A-FBE4-49A6-B6BA-B68B6E359698}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2F59859A-FBE4-49A6-B6BA-B68B6E359698}" name="Table1" displayName="Table1" ref="A2:B124" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A2:B124" xr:uid="{2F59859A-FBE4-49A6-B6BA-B68B6E359698}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:B3">
     <sortCondition ref="B2:B3"/>
   </sortState>
@@ -1167,7 +1173,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C799550E-49B1-4512-9CC1-86876BA1337E}">
-  <dimension ref="A1:B123"/>
+  <dimension ref="A1:B124"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="69.81640625" bestFit="1" customWidth="1"/>
@@ -1965,193 +1971,201 @@
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
-        <v>215</v>
+        <v>238</v>
       </c>
       <c r="B100" t="s">
-        <v>110</v>
+        <v>239</v>
       </c>
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B101" t="s">
-        <v>48</v>
+        <v>110</v>
       </c>
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B102" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A103" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B103" t="s">
-        <v>109</v>
+        <v>43</v>
       </c>
     </row>
     <row r="104" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A104" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B104" t="s">
-        <v>66</v>
+        <v>109</v>
       </c>
     </row>
     <row r="105" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A105" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B105" t="s">
-        <v>17</v>
+        <v>66</v>
       </c>
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A106" t="s">
-        <v>137</v>
+        <v>220</v>
       </c>
       <c r="B106" t="s">
-        <v>79</v>
+        <v>17</v>
       </c>
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
-        <v>221</v>
+        <v>137</v>
       </c>
       <c r="B107" t="s">
-        <v>6</v>
+        <v>79</v>
       </c>
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B108" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
     </row>
     <row r="109" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B109" t="s">
-        <v>68</v>
+        <v>19</v>
       </c>
     </row>
     <row r="110" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B110" t="s">
-        <v>42</v>
+        <v>68</v>
       </c>
     </row>
     <row r="111" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B111" t="s">
-        <v>84</v>
+        <v>42</v>
       </c>
     </row>
     <row r="112" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B112" t="s">
-        <v>11</v>
+        <v>84</v>
       </c>
     </row>
     <row r="113" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B113" t="s">
-        <v>104</v>
+        <v>11</v>
       </c>
     </row>
     <row r="114" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B114" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="115" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B115" t="s">
-        <v>93</v>
+        <v>106</v>
       </c>
     </row>
     <row r="116" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B116" t="s">
-        <v>59</v>
+        <v>93</v>
       </c>
     </row>
     <row r="117" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B117" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
     </row>
     <row r="118" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B118" t="s">
-        <v>10</v>
+        <v>69</v>
       </c>
     </row>
     <row r="119" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
-        <v>197</v>
+        <v>232</v>
       </c>
       <c r="B119" t="s">
-        <v>83</v>
+        <v>10</v>
       </c>
     </row>
     <row r="120" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
-        <v>233</v>
+        <v>197</v>
       </c>
       <c r="B120" t="s">
-        <v>26</v>
+        <v>83</v>
       </c>
     </row>
     <row r="121" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B121" t="s">
-        <v>47</v>
+        <v>26</v>
       </c>
     </row>
     <row r="122" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B122" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
     </row>
     <row r="123" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
+        <v>235</v>
+      </c>
+      <c r="B123" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A124" t="s">
         <v>236</v>
       </c>
-      <c r="B123" t="s">
+      <c r="B124" t="s">
         <v>108</v>
       </c>
     </row>

</xml_diff>